<commit_message>
fixed financial model download
</commit_message>
<xml_diff>
--- a/PROMPTly_Financial_Model.xlsx
+++ b/PROMPTly_Financial_Model.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Timothy\Documents\GitHub\promptly\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EEBCCBB-4334-4C36-98DC-B889D71E3CA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,10 +24,54 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+  <si>
+    <t>Metric</t>
+  </si>
+  <si>
+    <t>Units Sold (Monthly Pack)</t>
+  </si>
+  <si>
+    <t>Revenue</t>
+  </si>
+  <si>
+    <t>COGS</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Gross Profit</t>
+  </si>
+  <si>
+    <t>Gross Margin %</t>
+  </si>
+  <si>
+    <t>Operating Expenses</t>
+  </si>
+  <si>
+    <t>EBITDA</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="2">
+    <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
+    <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -49,8 +99,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="6" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +389,177 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="24" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6">
+        <v>2027</v>
+      </c>
+      <c r="C1" s="6">
+        <v>2028</v>
+      </c>
+      <c r="D1" s="6">
+        <v>2029</v>
+      </c>
+      <c r="E1" s="6">
+        <v>2030</v>
+      </c>
+      <c r="F1" s="6">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" s="1">
+        <v>2000</v>
+      </c>
+      <c r="D2" s="1">
+        <v>10000</v>
+      </c>
+      <c r="E2" s="1">
+        <v>36000</v>
+      </c>
+      <c r="F2" s="1">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="7">
+        <v>0</v>
+      </c>
+      <c r="C3" s="7">
+        <v>300000</v>
+      </c>
+      <c r="D3" s="7">
+        <v>1500000</v>
+      </c>
+      <c r="E3" s="7">
+        <v>5400000</v>
+      </c>
+      <c r="F3" s="7">
+        <v>15000000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="3">
+        <v>45</v>
+      </c>
+      <c r="D4" s="3">
+        <v>30</v>
+      </c>
+      <c r="E4" s="3">
+        <v>20</v>
+      </c>
+      <c r="F4" s="3">
+        <v>13.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="2">
+        <v>0</v>
+      </c>
+      <c r="C5" s="2">
+        <v>210000</v>
+      </c>
+      <c r="D5" s="2">
+        <v>1200000</v>
+      </c>
+      <c r="E5" s="2">
+        <v>4680000</v>
+      </c>
+      <c r="F5" s="2">
+        <v>13650000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="4">
+        <v>0</v>
+      </c>
+      <c r="C6" s="4">
+        <v>0.7</v>
+      </c>
+      <c r="D6" s="4">
+        <v>0.8</v>
+      </c>
+      <c r="E6" s="4">
+        <v>0.86</v>
+      </c>
+      <c r="F6" s="4">
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="2">
+        <v>400000</v>
+      </c>
+      <c r="C7" s="2">
+        <v>500000</v>
+      </c>
+      <c r="D7" s="2">
+        <v>1500000</v>
+      </c>
+      <c r="E7" s="2">
+        <v>3000000</v>
+      </c>
+      <c r="F7" s="2">
+        <v>7000000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="7">
+        <v>-400000</v>
+      </c>
+      <c r="C8" s="7">
+        <v>-290000</v>
+      </c>
+      <c r="D8" s="7">
+        <v>-300000</v>
+      </c>
+      <c r="E8" s="7">
+        <v>1680000</v>
+      </c>
+      <c r="F8" s="7">
+        <v>6650000</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>